<commit_message>
refocus on continuous phenotype mapping, drop the group labels entirely
</commit_message>
<xml_diff>
--- a/04_Figures/F01_phenotype/c_data/F01_phenotype_source_data.xlsx
+++ b/04_Figures/F01_phenotype/c_data/F01_phenotype_source_data.xlsx
@@ -7,59 +7,117 @@
   </bookViews>
   <sheets>
     <sheet name="overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="composite_modality" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="composite_structure" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="metadata" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="adaptation_space" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="change_over_training" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="phenotype_correlations" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="metadata" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t xml:space="preserve">sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">composite_modality</t>
-  </si>
-  <si>
-    <t xml:space="preserve">composite_structure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">best_g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bic_g1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bic_best</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bic_gain_over_g1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lrt_g1_vs_g2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lrt_p</t>
-  </si>
-  <si>
-    <t xml:space="preserve">agreement_with_label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E</t>
+    <t xml:space="preserve">adaptation_space</t>
+  </si>
+  <si>
+    <t xml:space="preserve">change_over_training</t>
+  </si>
+  <si>
+    <t xml:space="preserve">phenotype_correlations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">subject</t>
+  </si>
+  <si>
+    <t xml:space="preserve">given</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR_S03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR_S10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR_S16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR_S22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR_S24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR_S27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR_S28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR_S29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR_S04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR_S05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR_S06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR_S12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR_S14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR_S17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR_S21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR_S30</t>
   </si>
   <si>
     <t xml:space="preserve">trait</t>
   </si>
   <si>
-    <t xml:space="preserve">r</t>
-  </si>
-  <si>
-    <t xml:space="preserve">r2_alone</t>
+    <t xml:space="preserve">n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean_d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ci_lo_d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ci_hi_d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">moved</t>
   </si>
   <si>
     <t xml:space="preserve">d_fcsa_I</t>
@@ -86,6 +144,9 @@
     <t xml:space="preserve">d_1rm_ext</t>
   </si>
   <si>
+    <t xml:space="preserve">comp_hypertrophy</t>
+  </si>
+  <si>
     <t xml:space="preserve">volume_load</t>
   </si>
   <si>
@@ -98,55 +159,37 @@
     <t xml:space="preserve">figure</t>
   </si>
   <si>
-    <t xml:space="preserve">F01 responder phenotype and label construction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16 subjects, complete on every outcome except 1RM leg extension (15)</t>
+    <t xml:space="preserve">F01 the adaptation phenotypes, as continuous outcomes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16 subjects; 1RM leg extension has one missing value and drops that subject from its own cell only</t>
   </si>
   <si>
     <t xml:space="preserve">effect size</t>
   </si>
   <si>
-    <t xml:space="preserve">mean or group difference divided by the SD of the change score; 95% CI from the same t interval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">composite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">comp_hypertrophy arrives from the source spreadsheet without a stated formula; the five outcomes reconstruct it at r2 = 0.977</t>
-  </si>
-  <si>
-    <t xml:space="preserve">label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HR/LR is the exact median cut of comp_hypertrophy: the top eight are HR without exception</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bimodality</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mclust BIC selects two components; bootstrap LRT over 999 replicates gives p = 0.035, and that solution recovers the given label exactly (ARI = 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">internal flag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">an outcome with r2 &gt;= 0.20 against the composite is an ingredient of it and cannot corroborate the label cut from it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not claimed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">this figure reports the construction and the separations; it draws no inference about the proteomic result</t>
+    <t xml:space="preserve">mean change divided by the SD of the change score, with the 95% CI from the same t interval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a total, not a change, so it carries no row in panel A; it appears in the correlation structure and is tested like the rest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fibre counts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the MyoVision columns are fibre counts, not areas, despite the fCSA in their meta names; they move against area because larger fibres pack fewer into the imaged field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no group split</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the original HR/LR label appears in panel C only to show where a median cut would have fallen; nothing in this project now conditions on it</t>
   </si>
   <si>
     <t xml:space="preserve">source</t>
   </si>
   <si>
-    <t xml:space="preserve">03_Features/01_Responsiveness/c_data/01_label_audit.xlsx</t>
+    <t xml:space="preserve">00_input/c_data/phenotype.csv</t>
   </si>
 </sst>
 </file>
@@ -490,6 +533,11 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -503,54 +551,240 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="G1" t="s">
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="H1" t="s">
+      <c r="C2" t="n">
+        <v>-1.42304142922061</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.303907602765883</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-2.63475855869826</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.91761992678484</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="n">
-        <v>-118.837036895944</v>
-      </c>
-      <c r="D2" t="n">
-        <v>-116.370873414592</v>
-      </c>
-      <c r="E2" t="n">
-        <v>2.46616348135234</v>
-      </c>
-      <c r="F2" t="n">
-        <v>8.0113409258319</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-2.67204973175757</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.01108073336865</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.236734105650308</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.0222623115058</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-1.69691760964309</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-1.51250161478203</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-1.873864669413</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-1.73186407991361</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-1.35379612049505</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.423446018483994</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.392784170031834</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-0.0449439822378895</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.175348739400842</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.816121980025477</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-1.78949820048961</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-1.05401071162855</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2.32617092133602</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-0.877294199553262</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.922196975233213</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.824218361473447</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3.26065035749814</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.140642649809389</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.72310360799444</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-2.03590775812444</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3.55817426837434</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.0230984273437207</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1.84876317419805</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.70942169451657</v>
       </c>
     </row>
   </sheetData>
@@ -566,112 +800,236 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>28</v>
+      </c>
+      <c r="D1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="B2" t="n">
-        <v>0.856004310667277</v>
+        <v>16</v>
       </c>
       <c r="C2" t="n">
-        <v>0.732743379880961</v>
+        <v>1423.6646446056</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.106164398036218</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.639026784426162</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.426697988353726</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.67711459881652</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="n">
         <v>16</v>
       </c>
-      <c r="B3" t="n">
-        <v>0.829021879743861</v>
-      </c>
       <c r="C3" t="n">
-        <v>0.687277277094045</v>
+        <v>1330.43532202496</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0647222368306787</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-0.468140149559265</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.597584623220623</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.799239922163086</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="B4" t="n">
-        <v>0.835177563982897</v>
+        <v>16</v>
       </c>
       <c r="C4" t="n">
-        <v>0.697521563380406</v>
+        <v>1350.06906491591</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.0177310373388128</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.550593423728757</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.515131349051131</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.944395096260056</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.600282058411429</v>
+        <v>16</v>
       </c>
       <c r="C5" t="n">
-        <v>0.360338549650662</v>
+        <v>342.444977332126</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0998335565215276</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.433028829868416</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.632695942911471</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.695274924894311</v>
+      </c>
+      <c r="H5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.489823092226803</v>
+        <v>16</v>
       </c>
       <c r="C6" t="n">
-        <v>0.239926661678627</v>
+        <v>143.121029784818</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.110483414099061</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.422378972290883</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.643345800489004</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.664842150377003</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="B7" t="n">
-        <v>0.496807795570891</v>
+        <v>16</v>
       </c>
       <c r="C7" t="n">
-        <v>0.246817985740008</v>
+        <v>1.84624146014726</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.12495442488565</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.592092038495707</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.6578168112756</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.000423451596641191</v>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B8" t="n">
-        <v>0.273744611777964</v>
+        <v>16</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0749361124774681</v>
+        <v>31.6611618022249</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.35220874923773</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.819346362847788</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.88507113562768</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0000724683159868194</v>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B9" t="n">
-        <v>0.127677047329517</v>
+        <v>15</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0163014284147838</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" t="n">
-        <v>0.0433581560331737</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.00187992969459705</v>
+        <v>6.6246293696866</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.47932804284017</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.925546501275304</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.03310958440504</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0000520917471123112</v>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -687,82 +1045,462 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>42</v>
+      </c>
+      <c r="C1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" t="s">
-        <v>27</v>
+        <v>42</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.858823529411765</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.885294117647059</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.847058823529412</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.664705882352941</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-0.495953040816682</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.494117647058823</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.222879746194257</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.184257897693052</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.167647058823529</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" t="s">
-        <v>29</v>
+        <v>34</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.858823529411765</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.908823529411765</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.973529411764706</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.634290090777418</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.088235294117647</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.351293904597571</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-0.0590340837269001</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.0911764705882353</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" t="s">
-        <v>31</v>
+        <v>35</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.885294117647059</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.908823529411765</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.947058823529412</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.623529411764706</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-0.553348199842945</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.197058823529412</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.37638632635454</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.046511702330285</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.329411764705882</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" t="s">
-        <v>33</v>
+        <v>36</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.847058823529412</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.973529411764706</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.947058823529412</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.688235294117647</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-0.651950139708576</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.0323529411764706</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.370482227117607</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-0.00357782325617577</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.261764705882353</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-0.664705882352941</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.623529411764706</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.688235294117647</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.937454264095627</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-0.0911764705882353</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.165314778634151</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-0.189624632577316</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-0.0470588235294118</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-0.495953040816682</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-0.634290090777418</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-0.553348199842945</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.651950139708576</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.937454264095627</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.170713806334525</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.17134491313134</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-0.11459270482978</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-0.0721118664688944</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" t="s">
         <v>39</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.494117647058823</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.088235294117647</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.197058823529412</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0323529411764706</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.0911764705882353</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.170713806334525</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.0531368931324057</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.36314906050184</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.0470588235294118</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
         <v>40</v>
       </c>
-      <c r="B9" t="s">
-        <v>41</v>
+      <c r="B9" t="n">
+        <v>0.222879746194257</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.351293904597571</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.37638632635454</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.370482227117607</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.165314778634151</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.17134491313134</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.0531368931324057</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-0.389938523426517</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.330629557268302</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.184257897693052</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-0.0590340837269001</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.046511702330285</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-0.00357782325617577</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.189624632577316</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0.11459270482978</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.36314906050184</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-0.389938523426517</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.159213134899822</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
         <v>43</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.167647058823529</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0911764705882353</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.329411764705882</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.261764705882353</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.0470588235294118</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-0.0721118664688944</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.0470588235294118</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.330629557268302</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.159213134899822</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>